<commit_message>
fix:the dist to scr main
</commit_message>
<xml_diff>
--- a/Agile_Sprint_Plan_NGO_Events_MVP.xlsx
+++ b/Agile_Sprint_Plan_NGO_Events_MVP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trun Dada\Projects\Products\Evently\code\application\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2EBD45-8162-4133-BA0E-7E6AF6F76050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC81DEDA-E452-4DBE-8270-6CC6A754DBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary Dashboard" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="221">
   <si>
     <t>AGILE SPRINT PLAN — NGO Events Platform MVP</t>
   </si>
@@ -685,6 +685,9 @@
   </si>
   <si>
     <t>It will be same as like a CREATE EVENT (EVENTLY) project, but in this we have to add projects that will be of 2 year or more than a year.</t>
+  </si>
+  <si>
+    <t>Started</t>
   </si>
 </sst>
 </file>
@@ -923,14 +926,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1161,24 +1164,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -2395,16 +2398,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -2531,16 +2534,16 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
@@ -2641,16 +2644,16 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -2773,16 +2776,16 @@
       <c r="H18" s="3"/>
     </row>
     <row r="19" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="24"/>
     </row>
     <row r="20" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
@@ -5875,16 +5878,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -5976,7 +5979,7 @@
         <v>26</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>53</v>
+        <v>220</v>
       </c>
       <c r="F6" s="7">
         <v>3</v>
@@ -6011,16 +6014,16 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
@@ -6119,16 +6122,16 @@
       <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -6207,16 +6210,16 @@
       <c r="H16" s="3"/>
     </row>
     <row r="17" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -9323,16 +9326,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -9423,16 +9426,16 @@
       <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -9545,16 +9548,16 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -9623,16 +9626,16 @@
       <c r="H16" s="3"/>
     </row>
     <row r="17" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -10767,16 +10770,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -10847,16 +10850,16 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="22" t="s">
         <v>182</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="27"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="24"/>
     </row>
     <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -10969,16 +10972,16 @@
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="27"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -11051,16 +11054,16 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -11109,16 +11112,16 @@
       <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="24"/>
     </row>
     <row r="20" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
@@ -12219,12 +12222,12 @@
     <col min="1" max="1" width="37.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>216</v>
       </c>
@@ -12234,12 +12237,12 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>219</v>
       </c>

</xml_diff>